<commit_message>
methodology note implementated, legacy code removed
</commit_message>
<xml_diff>
--- a/data/keywords/statistics_gender/keyword_statistics_gender.xlsx
+++ b/data/keywords/statistics_gender/keyword_statistics_gender.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jojoa\OneDrive\Dokumente\OECD\RAnalysis\PRESS\data\keywords\statistics_gender\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/464195223dcae84f/Dokumente/OECD/RAnalysis/PRESS/data/keywords/statistics_gender/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75B125E7-729B-4A20-9583-A9FDE8F1370B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="13_ncr:1_{4958718D-BB12-46B8-B854-ED7C73E1CC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9866B986-64D3-4ACA-9E86-9A2E5E4BCBFB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="statistics" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="655" uniqueCount="589">
   <si>
     <t>id</t>
   </si>
@@ -766,9 +766,6 @@
     <t>indicador mdg</t>
   </si>
   <si>
-    <t>mdg-Indikator</t>
-  </si>
-  <si>
     <t>data standards</t>
   </si>
   <si>
@@ -826,9 +823,6 @@
     <t>monitoreo de los objetivos del milenio</t>
   </si>
   <si>
-    <t>mdg-Überwachung</t>
-  </si>
-  <si>
     <t>sdg monitoring</t>
   </si>
   <si>
@@ -838,9 +832,6 @@
     <t>monitoreo de los ods</t>
   </si>
   <si>
-    <t>sdg-Überwachung</t>
-  </si>
-  <si>
     <t>monitoring mdg</t>
   </si>
   <si>
@@ -850,9 +841,6 @@
     <t>monitories de los ddm</t>
   </si>
   <si>
-    <t>Überwachung von mdg</t>
-  </si>
-  <si>
     <t>monitoring sdg</t>
   </si>
   <si>
@@ -862,9 +850,6 @@
     <t>seguimiento de los ods</t>
   </si>
   <si>
-    <t>Überwachung von sdg</t>
-  </si>
-  <si>
     <t>release data</t>
   </si>
   <si>
@@ -898,9 +883,6 @@
     <t>seguimiento de los prsp</t>
   </si>
   <si>
-    <t>prsp-überwachung</t>
-  </si>
-  <si>
     <t>data revolution</t>
   </si>
   <si>
@@ -1042,9 +1024,6 @@
     <t>sistema estadístico nacional</t>
   </si>
   <si>
-    <t>nationalen statistischen Systems</t>
-  </si>
-  <si>
     <t>data linkage</t>
   </si>
   <si>
@@ -1192,9 +1171,6 @@
     <t>inteligencia artificial</t>
   </si>
   <si>
-    <t>künstliche Intellgenz</t>
-  </si>
-  <si>
     <t>machine learning</t>
   </si>
   <si>
@@ -1627,9 +1603,6 @@
     <t>desglose por sexo</t>
   </si>
   <si>
-    <t>Geschlechtertrennung</t>
-  </si>
-  <si>
     <t>gender index</t>
   </si>
   <si>
@@ -1693,9 +1666,6 @@
     <t>VBG</t>
   </si>
   <si>
-    <t>gbv</t>
-  </si>
-  <si>
     <t>VAW</t>
   </si>
   <si>
@@ -1705,12 +1675,6 @@
     <t>VCM</t>
   </si>
   <si>
-    <t>vaw</t>
-  </si>
-  <si>
-    <t>sdg5</t>
-  </si>
-  <si>
     <t>ODD5</t>
   </si>
   <si>
@@ -1744,9 +1708,6 @@
     <t>MGF</t>
   </si>
   <si>
-    <t>fgm</t>
-  </si>
-  <si>
     <t>SDSR</t>
   </si>
   <si>
@@ -1811,13 +1772,46 @@
   </si>
   <si>
     <t>vital registry</t>
+  </si>
+  <si>
+    <t>nationales statistisches System</t>
+  </si>
+  <si>
+    <t>prsp-Überwachung</t>
+  </si>
+  <si>
+    <t>geschlechtsspezifische Aufschlüsselung</t>
+  </si>
+  <si>
+    <t>MDG-Indikator</t>
+  </si>
+  <si>
+    <t>MDG-Überwachung</t>
+  </si>
+  <si>
+    <t>SDG-Überwachung</t>
+  </si>
+  <si>
+    <t>Überwachung von MDG</t>
+  </si>
+  <si>
+    <t>Überwachung von SDG</t>
+  </si>
+  <si>
+    <t>künstliche Intelligenz</t>
+  </si>
+  <si>
+    <t>Zensus</t>
+  </si>
+  <si>
+    <t>SDG5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1889,13 +1883,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF375623"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1918,7 +1905,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
@@ -1933,7 +1920,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2219,15 +2205,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E117"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="24.109375" customWidth="1"/>
-    <col min="3" max="3" width="32.109375" customWidth="1"/>
-    <col min="4" max="4" width="31.21875" customWidth="1"/>
-    <col min="5" max="5" width="30.5546875" customWidth="1"/>
+    <col min="1" max="1" width="4.6640625" customWidth="1"/>
+    <col min="2" max="2" width="24.1328125" customWidth="1"/>
+    <col min="3" max="3" width="32.1328125" customWidth="1"/>
+    <col min="4" max="4" width="31.19921875" customWidth="1"/>
+    <col min="5" max="5" width="30.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2238,13 +2225,13 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>0</v>
       </c>
@@ -2261,7 +2248,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2278,7 +2265,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2295,1776 +2282,1776 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A6">
         <v>3</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>17</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6">
+    <row r="7" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A7">
         <v>4</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B7" t="s">
         <v>20</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>21</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D7" t="s">
         <v>22</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7">
+    <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A8">
         <v>5</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B8" t="s">
         <v>24</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>25</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D8" t="s">
         <v>26</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>580</v>
-      </c>
-      <c r="C8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" t="s">
-        <v>30</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>583</v>
-      </c>
-      <c r="E9" s="7"/>
-    </row>
-    <row r="10" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>567</v>
+      </c>
+      <c r="C9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>6</v>
       </c>
       <c r="B10" t="s">
+        <v>570</v>
+      </c>
+      <c r="E10" s="7"/>
+    </row>
+    <row r="11" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A11">
+        <v>6</v>
+      </c>
+      <c r="B11" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>7</v>
-      </c>
-      <c r="B11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" t="s">
-        <v>34</v>
-      </c>
-      <c r="E11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>7</v>
       </c>
       <c r="B13" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A14">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D14" t="s">
-        <v>38</v>
-      </c>
-      <c r="E14" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>8</v>
       </c>
       <c r="B15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A16">
+        <v>8</v>
+      </c>
+      <c r="B16" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="14.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A17">
         <v>9</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>40</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C17" t="s">
         <v>41</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D17" t="s">
         <v>42</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E17" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17">
+    <row r="18" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A18">
         <v>10</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>44</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C18" t="s">
         <v>45</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D18" t="s">
         <v>46</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E18" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A18">
+    <row r="19" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A19">
         <v>11</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B19" t="s">
         <v>48</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C19" t="s">
         <v>49</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D19" t="s">
         <v>50</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E19" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19">
+    <row r="20" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A20">
         <v>12</v>
       </c>
-      <c r="B19" t="s">
-        <v>585</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A20">
+      <c r="B20" t="s">
+        <v>572</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A21">
         <v>11</v>
       </c>
-      <c r="B20" t="s">
-        <v>579</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A21">
+      <c r="B21" t="s">
+        <v>566</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A22">
         <v>12</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B22" t="s">
         <v>52</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C22" t="s">
         <v>53</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D22" t="s">
         <v>54</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E22" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A22">
+    <row r="23" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A23">
+        <v>12</v>
+      </c>
+      <c r="B23" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A24">
+        <v>12</v>
+      </c>
+      <c r="B24" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A25">
         <v>13</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B25" t="s">
         <v>56</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C25" t="s">
         <v>57</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D25" t="s">
         <v>58</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E25" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A23">
+    <row r="26" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A26">
         <v>14</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B26" t="s">
         <v>60</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C26" t="s">
         <v>61</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D26" t="s">
         <v>62</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E26" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A24">
+    <row r="27" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A27">
         <v>15</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B27" t="s">
         <v>64</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C27" t="s">
         <v>65</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D27" t="s">
         <v>66</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E27" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A25">
+    <row r="28" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A28">
         <v>16</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B28" t="s">
         <v>68</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C28" t="s">
         <v>69</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D28" t="s">
         <v>70</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E28" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A26">
+    <row r="29" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A29">
         <v>17</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B29" t="s">
         <v>72</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C29" t="s">
         <v>73</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D29" t="s">
         <v>74</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E29" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A27">
+    <row r="30" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A30">
         <v>18</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B30" t="s">
         <v>76</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C30" t="s">
         <v>77</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D30" t="s">
         <v>78</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E30" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A28">
+    <row r="31" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A31">
         <v>19</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B31" t="s">
         <v>80</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C31" t="s">
         <v>81</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D31" t="s">
         <v>82</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E31" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A29">
+    <row r="32" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A32">
         <v>20</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B32" t="s">
         <v>84</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C32" t="s">
         <v>85</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D32" t="s">
         <v>86</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E32" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A30">
+    <row r="33" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A33">
         <v>21</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B33" t="s">
         <v>88</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C33" t="s">
         <v>89</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D33" t="s">
         <v>90</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E33" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A31">
+    <row r="34" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A34">
         <v>22</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B34" t="s">
         <v>92</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C34" t="s">
         <v>93</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D34" t="s">
         <v>94</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E34" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A32">
+    <row r="35" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A35">
         <v>23</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B35" t="s">
         <v>96</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C35" t="s">
         <v>97</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D35" t="s">
         <v>98</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E35" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A33">
+    <row r="36" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A36">
         <v>24</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B36" t="s">
         <v>100</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C36" t="s">
         <v>100</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D36" t="s">
         <v>101</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E36" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A34">
+    <row r="37" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A37">
         <v>25</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B37" t="s">
         <v>103</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C37" t="s">
         <v>104</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D37" t="s">
         <v>105</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E37" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A35">
+    <row r="38" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A38">
         <v>26</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B38" t="s">
         <v>107</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C38" t="s">
         <v>108</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D38" t="s">
         <v>109</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E38" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A36">
+    <row r="39" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A39">
         <v>27</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B39" t="s">
         <v>111</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C39" t="s">
         <v>112</v>
       </c>
-      <c r="D36" t="s">
+      <c r="D39" t="s">
         <v>113</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E39" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A37">
+    <row r="40" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A40">
         <v>28</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B40" t="s">
         <v>115</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C40" t="s">
         <v>116</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D40" t="s">
         <v>117</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E40" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A38">
+    <row r="41" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A41">
         <v>29</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B41" t="s">
         <v>119</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C41" t="s">
         <v>120</v>
       </c>
-      <c r="D38" t="s">
+      <c r="D41" t="s">
         <v>121</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E41" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A39">
+    <row r="42" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A42">
         <v>30</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B42" t="s">
         <v>123</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C42" t="s">
         <v>124</v>
       </c>
-      <c r="D39" t="s">
+      <c r="D42" t="s">
         <v>125</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E42" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A40">
+    <row r="43" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A43">
         <v>31</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B43" t="s">
         <v>127</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C43" t="s">
         <v>128</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D43" t="s">
         <v>129</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E43" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A41">
+    <row r="44" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A44">
         <v>32</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B44" t="s">
         <v>131</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C44" t="s">
         <v>132</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D44" t="s">
         <v>133</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E44" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A42">
+    <row r="45" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A45">
         <v>32</v>
       </c>
-      <c r="B42" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A43">
+      <c r="B45" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A46">
         <v>32</v>
       </c>
-      <c r="B43" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A44">
+      <c r="B46" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A47">
         <v>33</v>
       </c>
-      <c r="B44" t="s">
-        <v>589</v>
-      </c>
-      <c r="C44" t="s">
+      <c r="B47" t="s">
+        <v>576</v>
+      </c>
+      <c r="C47" t="s">
         <v>136</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D47" t="s">
         <v>137</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E47" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A45">
+    <row r="48" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A48">
         <v>33</v>
       </c>
-      <c r="B45" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A46">
+      <c r="B48" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A49">
         <v>33</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B49" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A47">
+    <row r="50" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A50">
         <v>34</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B50" t="s">
         <v>139</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C50" t="s">
         <v>140</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D50" t="s">
         <v>141</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E50" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A48">
+    <row r="51" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A51">
         <v>35</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B51" t="s">
         <v>143</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C51" t="s">
         <v>144</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D51" t="s">
         <v>145</v>
       </c>
-      <c r="E48" t="s">
+      <c r="E51" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A49">
+    <row r="52" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A52">
         <v>36</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B52" t="s">
         <v>147</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C52" t="s">
         <v>148</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D52" t="s">
         <v>149</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E52" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A50">
+    <row r="53" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A53">
         <v>37</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B53" t="s">
         <v>151</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C53" t="s">
         <v>152</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D53" t="s">
         <v>153</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E53" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A51">
+    <row r="54" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A54">
         <v>37</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D54" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A52">
+    <row r="55" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A55">
         <v>38</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B55" t="s">
         <v>156</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C55" t="s">
         <v>157</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D55" t="s">
         <v>158</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E55" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A53">
+    <row r="56" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A56">
         <v>38</v>
       </c>
-      <c r="D53" t="s">
+      <c r="D56" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A54">
+    <row r="57" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A57">
         <v>39</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B57" t="s">
         <v>161</v>
       </c>
-      <c r="C54" t="s">
+      <c r="C57" t="s">
         <v>162</v>
       </c>
-      <c r="D54" t="s">
+      <c r="D57" t="s">
         <v>163</v>
       </c>
-      <c r="E54" t="s">
+      <c r="E57" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A55">
+    <row r="58" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A58">
         <v>40</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B58" t="s">
         <v>165</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C58" t="s">
         <v>166</v>
       </c>
-      <c r="D55" t="s">
+      <c r="D58" t="s">
         <v>167</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E58" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A56">
+    <row r="59" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A59">
         <v>41</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B59" t="s">
         <v>169</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C59" t="s">
         <v>170</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D59" t="s">
         <v>171</v>
       </c>
-      <c r="E56" t="s">
+      <c r="E59" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A57">
+    <row r="60" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A60">
         <v>42</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B60" t="s">
         <v>173</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C60" t="s">
         <v>174</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D60" t="s">
         <v>175</v>
       </c>
-      <c r="E57" t="s">
+      <c r="E60" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A58">
+    <row r="61" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A61">
         <v>43</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B61" t="s">
         <v>177</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C61" t="s">
         <v>178</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D61" t="s">
         <v>179</v>
       </c>
-      <c r="E58" t="s">
+      <c r="E61" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A59">
+    <row r="62" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A62">
         <v>44</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B62" t="s">
         <v>181</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C62" t="s">
         <v>182</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D62" t="s">
         <v>183</v>
       </c>
-      <c r="E59" t="s">
+      <c r="E62" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A60">
+    <row r="63" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A63">
         <v>45</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B63" t="s">
         <v>185</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C63" t="s">
         <v>186</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D63" t="s">
         <v>187</v>
       </c>
-      <c r="E60" t="s">
+      <c r="E63" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A61">
+    <row r="64" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A64">
         <v>46</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B64" t="s">
         <v>189</v>
       </c>
-      <c r="C61" t="s">
+      <c r="C64" t="s">
         <v>190</v>
       </c>
-      <c r="D61" t="s">
+      <c r="D64" t="s">
         <v>191</v>
       </c>
-      <c r="E61" t="s">
+      <c r="E64" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A62">
+    <row r="65" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A65">
         <v>47</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B65" t="s">
         <v>193</v>
-      </c>
-      <c r="C62" t="s">
-        <v>194</v>
-      </c>
-      <c r="D62" t="s">
-        <v>195</v>
-      </c>
-      <c r="E62" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A63">
-        <v>48</v>
-      </c>
-      <c r="B63" t="s">
-        <v>197</v>
-      </c>
-      <c r="C63" t="s">
-        <v>198</v>
-      </c>
-      <c r="D63" t="s">
-        <v>199</v>
-      </c>
-      <c r="E63" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A64">
-        <v>49</v>
-      </c>
-      <c r="B64" t="s">
-        <v>201</v>
-      </c>
-      <c r="C64" t="s">
-        <v>202</v>
-      </c>
-      <c r="D64" t="s">
-        <v>203</v>
-      </c>
-      <c r="E64" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A65">
-        <v>50</v>
-      </c>
-      <c r="B65" t="s">
-        <v>205</v>
       </c>
       <c r="C65" t="s">
         <v>194</v>
       </c>
       <c r="D65" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="E65" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A66">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B66" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="C66" t="s">
         <v>198</v>
       </c>
       <c r="D66" t="s">
+        <v>199</v>
+      </c>
+      <c r="E66" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A67">
+        <v>49</v>
+      </c>
+      <c r="B67" t="s">
+        <v>201</v>
+      </c>
+      <c r="C67" t="s">
+        <v>202</v>
+      </c>
+      <c r="D67" t="s">
+        <v>203</v>
+      </c>
+      <c r="E67" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A68">
+        <v>50</v>
+      </c>
+      <c r="B68" t="s">
+        <v>205</v>
+      </c>
+      <c r="C68" t="s">
+        <v>194</v>
+      </c>
+      <c r="D68" t="s">
+        <v>206</v>
+      </c>
+      <c r="E68" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A69">
+        <v>51</v>
+      </c>
+      <c r="B69" t="s">
+        <v>208</v>
+      </c>
+      <c r="C69" t="s">
+        <v>198</v>
+      </c>
+      <c r="D69" t="s">
         <v>209</v>
       </c>
-      <c r="E66" t="s">
+      <c r="E69" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A67">
+    <row r="70" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A70">
         <v>52</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B70" t="s">
         <v>211</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C70" t="s">
         <v>212</v>
       </c>
-      <c r="D67" t="s">
+      <c r="D70" t="s">
         <v>213</v>
       </c>
-      <c r="E67" t="s">
+      <c r="E70" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A68">
+    <row r="71" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A71">
         <v>53</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B71" t="s">
         <v>215</v>
       </c>
-      <c r="C68" t="s">
+      <c r="C71" t="s">
         <v>216</v>
       </c>
-      <c r="D68" t="s">
+      <c r="D71" t="s">
         <v>217</v>
       </c>
-      <c r="E68" t="s">
+      <c r="E71" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A69">
+    <row r="72" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A72">
         <v>54</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B72" t="s">
         <v>219</v>
       </c>
-      <c r="C69" t="s">
+      <c r="C72" t="s">
         <v>220</v>
       </c>
-      <c r="D69" t="s">
+      <c r="D72" t="s">
         <v>221</v>
       </c>
-      <c r="E69" t="s">
+      <c r="E72" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A70">
+    <row r="73" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A73">
         <v>55</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B73" t="s">
         <v>223</v>
       </c>
-      <c r="C70" t="s">
+      <c r="C73" t="s">
         <v>224</v>
       </c>
-      <c r="D70" t="s">
+      <c r="D73" t="s">
         <v>225</v>
       </c>
-      <c r="E70" t="s">
+      <c r="E73" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A71">
+    <row r="74" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A74">
         <v>56</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B74" t="s">
         <v>227</v>
       </c>
-      <c r="C71" t="s">
+      <c r="C74" t="s">
         <v>228</v>
       </c>
-      <c r="D71" t="s">
+      <c r="D74" t="s">
         <v>229</v>
       </c>
-      <c r="E71" t="s">
+      <c r="E74" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A72">
+    <row r="75" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A75">
         <v>57</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B75" t="s">
         <v>231</v>
       </c>
-      <c r="C72" t="s">
+      <c r="C75" t="s">
         <v>232</v>
       </c>
-      <c r="D72" t="s">
+      <c r="D75" t="s">
         <v>233</v>
       </c>
-      <c r="E72" t="s">
+      <c r="E75" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="73" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A73">
+    <row r="76" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A76">
         <v>58</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B76" t="s">
         <v>235</v>
       </c>
-      <c r="C73" t="s">
+      <c r="C76" t="s">
         <v>236</v>
       </c>
-      <c r="D73" t="s">
+      <c r="D76" t="s">
         <v>237</v>
       </c>
-      <c r="E73" t="s">
+      <c r="E76" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="74" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A74">
+    <row r="77" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A77">
         <v>59</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B77" t="s">
         <v>239</v>
       </c>
-      <c r="C74" t="s">
+      <c r="C77" t="s">
         <v>240</v>
       </c>
-      <c r="D74" t="s">
+      <c r="D77" t="s">
         <v>241</v>
       </c>
-      <c r="E74" t="s">
+      <c r="E77" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A78">
+        <v>60</v>
+      </c>
+      <c r="B78" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A75">
-        <v>60</v>
-      </c>
-      <c r="B75" t="s">
+      <c r="C78" t="s">
         <v>243</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D78" t="s">
         <v>244</v>
       </c>
-      <c r="D75" t="s">
+      <c r="E78" t="s">
         <v>245</v>
       </c>
-      <c r="E75" t="s">
+    </row>
+    <row r="79" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A79">
+        <v>61</v>
+      </c>
+      <c r="B79" t="s">
         <v>246</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A76">
-        <v>61</v>
-      </c>
-      <c r="B76" t="s">
+      <c r="C79" t="s">
         <v>247</v>
       </c>
-      <c r="C76" t="s">
+      <c r="D79" t="s">
         <v>248</v>
       </c>
-      <c r="D76" t="s">
+      <c r="E79" t="s">
         <v>249</v>
       </c>
-      <c r="E76" t="s">
+    </row>
+    <row r="80" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A80">
+        <v>62</v>
+      </c>
+      <c r="B80" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A77">
-        <v>62</v>
-      </c>
-      <c r="B77" t="s">
+      <c r="C80" t="s">
         <v>251</v>
       </c>
-      <c r="C77" t="s">
+      <c r="D80" t="s">
         <v>252</v>
       </c>
-      <c r="D77" t="s">
+      <c r="E80" t="s">
         <v>253</v>
       </c>
-      <c r="E77" t="s">
+    </row>
+    <row r="81" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A81">
+        <v>63</v>
+      </c>
+      <c r="B81" t="s">
         <v>254</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A78">
-        <v>63</v>
-      </c>
-      <c r="B78" t="s">
+      <c r="C81" t="s">
         <v>255</v>
       </c>
-      <c r="C78" t="s">
+      <c r="D81" t="s">
         <v>256</v>
       </c>
-      <c r="D78" t="s">
+      <c r="E81" t="s">
         <v>257</v>
       </c>
-      <c r="E78" t="s">
+    </row>
+    <row r="82" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A82">
+        <v>64</v>
+      </c>
+      <c r="B82" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A79">
-        <v>64</v>
-      </c>
-      <c r="B79" t="s">
+      <c r="C82" t="s">
         <v>259</v>
       </c>
-      <c r="C79" t="s">
+      <c r="D82" t="s">
         <v>260</v>
       </c>
-      <c r="D79" t="s">
+      <c r="E82" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A83">
+        <v>65</v>
+      </c>
+      <c r="B83" t="s">
         <v>261</v>
       </c>
-      <c r="E79" t="s">
+      <c r="C83" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A80">
-        <v>65</v>
-      </c>
-      <c r="B80" t="s">
+      <c r="D83" t="s">
         <v>263</v>
       </c>
-      <c r="C80" t="s">
+      <c r="E83" t="s">
+        <v>583</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A84">
+        <v>66</v>
+      </c>
+      <c r="B84" t="s">
         <v>264</v>
       </c>
-      <c r="D80" t="s">
+      <c r="C84" t="s">
         <v>265</v>
       </c>
-      <c r="E80" t="s">
+      <c r="D84" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A81">
-        <v>66</v>
-      </c>
-      <c r="B81" t="s">
+      <c r="E84" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A85">
+        <v>67</v>
+      </c>
+      <c r="B85" t="s">
         <v>267</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C85" t="s">
         <v>268</v>
       </c>
-      <c r="D81" t="s">
+      <c r="D85" t="s">
         <v>269</v>
       </c>
-      <c r="E81" t="s">
+      <c r="E85" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A86">
+        <v>68</v>
+      </c>
+      <c r="B86" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A82">
-        <v>67</v>
-      </c>
-      <c r="B82" t="s">
+      <c r="C86" t="s">
         <v>271</v>
       </c>
-      <c r="C82" t="s">
+      <c r="D86" t="s">
         <v>272</v>
       </c>
-      <c r="D82" t="s">
+      <c r="E86" t="s">
         <v>273</v>
       </c>
-      <c r="E82" t="s">
+    </row>
+    <row r="87" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A87">
+        <v>69</v>
+      </c>
+      <c r="B87" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A83">
-        <v>68</v>
-      </c>
-      <c r="B83" t="s">
+      <c r="C87" t="s">
         <v>275</v>
       </c>
-      <c r="C83" t="s">
+      <c r="D87" t="s">
         <v>276</v>
       </c>
-      <c r="D83" t="s">
+      <c r="E87" t="s">
         <v>277</v>
       </c>
-      <c r="E83" t="s">
+    </row>
+    <row r="88" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A88">
+        <v>70</v>
+      </c>
+      <c r="B88" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A84">
-        <v>69</v>
-      </c>
-      <c r="B84" t="s">
+      <c r="C88" t="s">
         <v>279</v>
       </c>
-      <c r="C84" t="s">
+      <c r="D88" t="s">
         <v>280</v>
       </c>
-      <c r="D84" t="s">
+      <c r="E88" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A89">
+        <v>71</v>
+      </c>
+      <c r="B89" t="s">
         <v>281</v>
       </c>
-      <c r="E84" t="s">
+      <c r="C89" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A85">
-        <v>70</v>
-      </c>
-      <c r="B85" t="s">
+      <c r="D89" t="s">
         <v>283</v>
       </c>
-      <c r="C85" t="s">
+      <c r="E89" t="s">
         <v>284</v>
       </c>
-      <c r="D85" t="s">
+    </row>
+    <row r="90" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A90">
+        <v>72</v>
+      </c>
+      <c r="B90" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="E85" t="s">
+      <c r="C90" s="3" t="s">
         <v>286</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A86">
-        <v>71</v>
-      </c>
-      <c r="B86" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A87">
-        <v>71</v>
-      </c>
-      <c r="B87" t="s">
+      <c r="D90" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="E90" s="5" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A91">
+        <v>73</v>
+      </c>
+      <c r="B91" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="E91" s="5" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A92">
+        <v>74</v>
+      </c>
+      <c r="B92" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="E92" s="5" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A93">
+        <v>75</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="E93" s="5" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A94">
+        <v>76</v>
+      </c>
+      <c r="B94" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="E94" s="5" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A95">
+        <v>77</v>
+      </c>
+      <c r="B95" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="E95" s="5" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A96">
+        <v>78</v>
+      </c>
+      <c r="B96" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="E96" s="5" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A97">
+        <v>79</v>
+      </c>
+      <c r="B97" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A98">
+        <v>80</v>
+      </c>
+      <c r="B98" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="D98" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A99">
+        <v>81</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C99" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="E99" s="5" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A100">
+        <v>82</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>323</v>
+      </c>
+      <c r="E100" s="5" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A101">
+        <v>83</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>326</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="E101" s="5" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A102">
+        <v>84</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>329</v>
+      </c>
+      <c r="D102" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="E102" s="5" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A103">
+        <v>85</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="C103" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>376</v>
+      </c>
+      <c r="E103" s="9" t="s">
         <v>586</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A88">
-        <v>71</v>
-      </c>
-      <c r="B88" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A89">
-        <v>72</v>
-      </c>
-      <c r="B89" t="s">
-        <v>287</v>
-      </c>
-      <c r="C89" t="s">
-        <v>288</v>
-      </c>
-      <c r="D89" t="s">
-        <v>289</v>
-      </c>
-      <c r="E89" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A90">
-        <v>73</v>
-      </c>
-      <c r="B90" s="3" t="s">
-        <v>291</v>
-      </c>
-      <c r="C90" s="3" t="s">
-        <v>292</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="E90" s="5" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A91">
-        <v>74</v>
-      </c>
-      <c r="B91" s="3" t="s">
-        <v>295</v>
-      </c>
-      <c r="C91" s="3" t="s">
-        <v>296</v>
-      </c>
-      <c r="D91" s="3" t="s">
-        <v>297</v>
-      </c>
-      <c r="E91" s="5" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A92">
-        <v>75</v>
-      </c>
-      <c r="B92" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="C92" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="D92" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="E92" s="5" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A93">
-        <v>76</v>
-      </c>
-      <c r="B93" s="3" t="s">
-        <v>303</v>
-      </c>
-      <c r="C93" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="D93" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="E93" s="5" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A94">
-        <v>77</v>
-      </c>
-      <c r="B94" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="C94" s="3" t="s">
-        <v>307</v>
-      </c>
-      <c r="D94" s="3" t="s">
-        <v>308</v>
-      </c>
-      <c r="E94" s="5" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A95">
-        <v>78</v>
-      </c>
-      <c r="B95" s="3" t="s">
-        <v>310</v>
-      </c>
-      <c r="C95" s="3" t="s">
-        <v>311</v>
-      </c>
-      <c r="D95" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="E95" s="5" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A96">
-        <v>79</v>
-      </c>
-      <c r="B96" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="C96" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="D96" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="E96" s="5" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A97">
-        <v>80</v>
-      </c>
-      <c r="B97" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>318</v>
-      </c>
-      <c r="D97" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="E97" s="5" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A98">
-        <v>81</v>
-      </c>
-      <c r="B98" s="3" t="s">
-        <v>321</v>
-      </c>
-      <c r="C98" s="3" t="s">
-        <v>322</v>
-      </c>
-      <c r="D98" s="3" t="s">
-        <v>323</v>
-      </c>
-      <c r="E98" s="5" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A99">
-        <v>82</v>
-      </c>
-      <c r="B99" s="3" t="s">
-        <v>325</v>
-      </c>
-      <c r="C99" s="3" t="s">
-        <v>326</v>
-      </c>
-      <c r="D99" s="3" t="s">
-        <v>327</v>
-      </c>
-      <c r="E99" s="5" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A100">
-        <v>83</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="C100" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="D100" s="3" t="s">
-        <v>329</v>
-      </c>
-      <c r="E100" s="5" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A101">
-        <v>84</v>
-      </c>
-      <c r="B101" s="3" t="s">
-        <v>331</v>
-      </c>
-      <c r="C101" s="3" t="s">
-        <v>332</v>
-      </c>
-      <c r="D101" s="3" t="s">
-        <v>333</v>
-      </c>
-      <c r="E101" s="5" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A102">
-        <v>85</v>
-      </c>
-      <c r="B102" s="3" t="s">
-        <v>335</v>
-      </c>
-      <c r="C102" s="3" t="s">
-        <v>336</v>
-      </c>
-      <c r="D102" s="3" t="s">
-        <v>337</v>
-      </c>
-      <c r="E102" s="5" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A103">
+    <row r="104" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A104">
         <v>86</v>
       </c>
-      <c r="B103" s="3" t="s">
+      <c r="B104" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="D104" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="E104" s="9" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A105">
+        <v>87</v>
+      </c>
+      <c r="B105" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="C103" s="3" t="s">
+      <c r="C105" s="3" t="s">
         <v>382</v>
       </c>
-      <c r="D103" s="3" t="s">
+      <c r="D105" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="E103" s="10" t="s">
+      <c r="E105" s="9" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="104" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A104">
-        <v>87</v>
-      </c>
-      <c r="B104" s="3" t="s">
+    <row r="106" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A106">
+        <v>88</v>
+      </c>
+      <c r="B106" s="3" t="s">
         <v>385</v>
       </c>
-      <c r="C104" s="3" t="s">
+      <c r="C106" s="3" t="s">
         <v>386</v>
       </c>
-      <c r="D104" s="3" t="s">
+      <c r="D106" s="3" t="s">
         <v>387</v>
       </c>
-      <c r="E104" s="9" t="s">
+      <c r="E106" s="9" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="105" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A105">
+    <row r="107" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A107" s="8">
         <v>88</v>
-      </c>
-      <c r="B105" s="3" t="s">
-        <v>389</v>
-      </c>
-      <c r="C105" s="3" t="s">
-        <v>390</v>
-      </c>
-      <c r="D105" s="3" t="s">
-        <v>391</v>
-      </c>
-      <c r="E105" s="9" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A106">
-        <v>89</v>
-      </c>
-      <c r="B106" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="C106" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="D106" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="E106" s="9" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A107" s="8">
-        <v>89</v>
       </c>
       <c r="B107" s="3"/>
       <c r="C107" s="3" t="s">
-        <v>397</v>
+        <v>389</v>
       </c>
       <c r="D107" s="3"/>
       <c r="E107" s="9"/>
     </row>
-    <row r="108" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A108" s="8">
+        <v>89</v>
+      </c>
+      <c r="B108" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="C108" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="D108" s="8" t="s">
+        <v>391</v>
+      </c>
+      <c r="E108" s="8" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A109" s="8">
         <v>90</v>
       </c>
-      <c r="B108" s="8" t="s">
-        <v>329</v>
-      </c>
-      <c r="C108" s="8" t="s">
+      <c r="B109" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="C109" s="8" t="s">
+        <v>392</v>
+      </c>
+      <c r="D109" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="E109" s="8" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A110" s="8">
+        <v>91</v>
+      </c>
+      <c r="B110" s="8" t="s">
+        <v>395</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>396</v>
+      </c>
+      <c r="D110" s="8" t="s">
+        <v>397</v>
+      </c>
+      <c r="E110" s="8" t="s">
         <v>398</v>
       </c>
-      <c r="D108" s="8" t="s">
+    </row>
+    <row r="111" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A111" s="8">
+        <v>92</v>
+      </c>
+      <c r="B111" s="8" t="s">
         <v>399</v>
       </c>
-      <c r="E108" s="8" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="8">
-        <v>91</v>
-      </c>
-      <c r="B109" s="8" t="s">
+      <c r="C111" s="8" t="s">
         <v>400</v>
       </c>
-      <c r="C109" s="8" t="s">
-        <v>400</v>
-      </c>
-      <c r="D109" s="8" t="s">
+      <c r="D111" s="8" t="s">
         <v>401</v>
       </c>
-      <c r="E109" s="8" t="s">
+      <c r="E111" s="8" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="110" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="8">
-        <v>92</v>
-      </c>
-      <c r="B110" s="8" t="s">
+    <row r="112" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A112" s="8">
+        <v>93</v>
+      </c>
+      <c r="B112" s="3" t="s">
         <v>403</v>
       </c>
-      <c r="C110" s="8" t="s">
+      <c r="C112" s="3" t="s">
         <v>404</v>
       </c>
-      <c r="D110" s="8" t="s">
+      <c r="D112" s="3" t="s">
         <v>405</v>
       </c>
-      <c r="E110" s="8" t="s">
+      <c r="E112" s="9" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="111" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="8">
-        <v>93</v>
-      </c>
-      <c r="B111" s="8" t="s">
+    <row r="113" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A113" s="8">
+        <v>94</v>
+      </c>
+      <c r="B113" s="8" t="s">
         <v>407</v>
       </c>
-      <c r="C111" s="8" t="s">
+      <c r="C113" s="8" t="s">
         <v>408</v>
       </c>
-      <c r="D111" s="8" t="s">
+      <c r="D113" s="8" t="s">
         <v>409</v>
       </c>
-      <c r="E111" s="8" t="s">
+      <c r="E113" s="8" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="112" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A112" s="8">
-        <v>94</v>
-      </c>
-      <c r="B112" s="3" t="s">
+    <row r="114" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A114" s="8">
+        <v>95</v>
+      </c>
+      <c r="B114" s="8" t="s">
         <v>411</v>
       </c>
-      <c r="C112" s="3" t="s">
+      <c r="C114" s="8" t="s">
         <v>412</v>
       </c>
-      <c r="D112" s="3" t="s">
+      <c r="D114" s="8" t="s">
         <v>413</v>
       </c>
-      <c r="E112" s="9" t="s">
+      <c r="E114" s="8" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="113" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="8">
-        <v>95</v>
-      </c>
-      <c r="B113" s="8" t="s">
+    <row r="115" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A115" s="8">
+        <v>96</v>
+      </c>
+      <c r="B115" s="8" t="s">
+        <v>377</v>
+      </c>
+      <c r="C115" s="8" t="s">
         <v>415</v>
       </c>
-      <c r="C113" s="8" t="s">
+      <c r="D115" s="8" t="s">
+        <v>379</v>
+      </c>
+      <c r="E115" s="8" t="s">
         <v>416</v>
       </c>
-      <c r="D113" s="8" t="s">
-        <v>417</v>
-      </c>
-      <c r="E113" s="8" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="114" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="8">
-        <v>96</v>
-      </c>
-      <c r="B114" s="8" t="s">
-        <v>419</v>
-      </c>
-      <c r="C114" s="8" t="s">
-        <v>420</v>
-      </c>
-      <c r="D114" s="8" t="s">
-        <v>421</v>
-      </c>
-      <c r="E114" s="8" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="8">
+    </row>
+    <row r="116" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A116" s="8">
         <v>97</v>
       </c>
-      <c r="B115" s="8" t="s">
-        <v>385</v>
-      </c>
-      <c r="C115" s="8" t="s">
-        <v>423</v>
-      </c>
-      <c r="D115" s="8" t="s">
-        <v>387</v>
-      </c>
-      <c r="E115" s="8" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A116" s="8">
+      <c r="B116" s="8" t="s">
+        <v>558</v>
+      </c>
+      <c r="C116" s="8" t="s">
+        <v>559</v>
+      </c>
+      <c r="D116" s="8" t="s">
+        <v>560</v>
+      </c>
+      <c r="E116" s="8" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A117" s="8">
         <v>98</v>
       </c>
-      <c r="B116" s="8" t="s">
-        <v>571</v>
-      </c>
-      <c r="C116" s="8" t="s">
-        <v>572</v>
-      </c>
-      <c r="D116" s="8" t="s">
-        <v>573</v>
-      </c>
-      <c r="E116" s="8" t="s">
-        <v>574</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A117" s="8">
-        <v>99</v>
-      </c>
       <c r="B117" s="8" t="s">
-        <v>575</v>
+        <v>562</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>576</v>
-      </c>
-      <c r="D117" s="11" t="s">
-        <v>577</v>
+        <v>563</v>
+      </c>
+      <c r="D117" s="10" t="s">
+        <v>564</v>
       </c>
       <c r="E117" s="8" t="s">
-        <v>578</v>
+        <v>565</v>
       </c>
     </row>
   </sheetData>
@@ -4076,15 +4063,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9878D5F-0194-4AC6-B566-F63E204E3C96}">
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="17.77734375" customWidth="1"/>
-    <col min="3" max="3" width="16.44140625" customWidth="1"/>
-    <col min="4" max="4" width="11.44140625" customWidth="1"/>
-    <col min="5" max="5" width="19.44140625" customWidth="1"/>
+    <col min="2" max="2" width="17.796875" customWidth="1"/>
+    <col min="3" max="3" width="16.46484375" customWidth="1"/>
+    <col min="4" max="4" width="11.46484375" customWidth="1"/>
+    <col min="5" max="5" width="19.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4095,233 +4082,233 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="C2" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="D2" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
       <c r="E2" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="C3" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="D3" t="s">
-        <v>342</v>
+        <v>335</v>
       </c>
       <c r="E3" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="C4" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="D4" t="s">
-        <v>343</v>
+        <v>336</v>
       </c>
       <c r="E4" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="C5" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="D5" t="s">
-        <v>344</v>
+        <v>337</v>
       </c>
       <c r="E5" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="C6" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="D6" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
       <c r="E6" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>346</v>
+        <v>339</v>
       </c>
       <c r="C7" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="D7" t="s">
-        <v>348</v>
+        <v>341</v>
       </c>
       <c r="E7" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="C8" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="D8" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="E8" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="C9" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="D9" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="E9" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="C10" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="D10" t="s">
-        <v>355</v>
+        <v>348</v>
       </c>
       <c r="E10" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="C11" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="D11" t="s">
-        <v>356</v>
+        <v>349</v>
       </c>
       <c r="E11" t="s">
-        <v>356</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="5"/>
     </row>
-    <row r="14" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>12</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>425</v>
+        <v>417</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="E14" s="9"/>
     </row>
-    <row r="15" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>427</v>
+        <v>419</v>
       </c>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
     </row>
-    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>428</v>
+        <v>420</v>
       </c>
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
@@ -4335,14 +4322,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09178084-6EE9-4A4A-ACE4-85554F1DA5DB}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="3" width="13.5546875" customWidth="1"/>
-    <col min="4" max="4" width="17.88671875" customWidth="1"/>
-    <col min="5" max="5" width="20.5546875" customWidth="1"/>
+    <col min="3" max="3" width="13.53125" customWidth="1"/>
+    <col min="4" max="4" width="17.86328125" customWidth="1"/>
+    <col min="5" max="5" width="20.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -4353,111 +4340,111 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
       <c r="C2" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="D2" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="E2" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>364</v>
+        <v>357</v>
       </c>
       <c r="C4" t="s">
-        <v>365</v>
+        <v>358</v>
       </c>
       <c r="D4" t="s">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="E4" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>368</v>
+        <v>361</v>
       </c>
       <c r="C5" t="s">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="D5" t="s">
-        <v>370</v>
+        <v>363</v>
       </c>
       <c r="E5" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="C7" t="s">
-        <v>374</v>
+        <v>367</v>
       </c>
       <c r="D7" t="s">
-        <v>375</v>
+        <v>368</v>
       </c>
       <c r="E7" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
       <c r="C8" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
       <c r="D8" t="s">
-        <v>379</v>
+        <v>372</v>
       </c>
       <c r="E8" t="s">
-        <v>380</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>
@@ -4468,15 +4455,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B779B73F-545A-4F4D-8CFE-66FFC11C3D0C}">
   <dimension ref="A1:E32"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="31.88671875" customWidth="1"/>
-    <col min="4" max="4" width="32.109375" customWidth="1"/>
+    <col min="3" max="3" width="31.86328125" customWidth="1"/>
+    <col min="4" max="4" width="32.1328125" customWidth="1"/>
     <col min="5" max="5" width="39" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -4487,537 +4474,537 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>429</v>
+        <v>421</v>
       </c>
       <c r="C2" t="s">
-        <v>430</v>
+        <v>422</v>
       </c>
       <c r="D2" t="s">
-        <v>431</v>
+        <v>423</v>
       </c>
       <c r="E2" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>433</v>
+        <v>425</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>434</v>
+        <v>426</v>
       </c>
       <c r="D3" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="E3" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>437</v>
+        <v>429</v>
       </c>
       <c r="C4" t="s">
-        <v>438</v>
+        <v>430</v>
       </c>
       <c r="D4" t="s">
-        <v>439</v>
+        <v>431</v>
       </c>
       <c r="E4" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>441</v>
+        <v>433</v>
       </c>
       <c r="C5" t="s">
-        <v>442</v>
+        <v>434</v>
       </c>
       <c r="D5" t="s">
-        <v>443</v>
+        <v>435</v>
       </c>
       <c r="E5" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
       <c r="C6" t="s">
-        <v>446</v>
+        <v>438</v>
       </c>
       <c r="D6" t="s">
-        <v>447</v>
+        <v>439</v>
       </c>
       <c r="E6" t="s">
-        <v>570</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>448</v>
+        <v>440</v>
       </c>
       <c r="C7" t="s">
-        <v>449</v>
+        <v>441</v>
       </c>
       <c r="D7" t="s">
-        <v>450</v>
+        <v>442</v>
       </c>
       <c r="E7" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>452</v>
+        <v>444</v>
       </c>
       <c r="C8" t="s">
-        <v>453</v>
+        <v>445</v>
       </c>
       <c r="D8" t="s">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="E8" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>456</v>
+        <v>448</v>
       </c>
       <c r="C9" t="s">
-        <v>457</v>
+        <v>449</v>
       </c>
       <c r="D9" t="s">
-        <v>458</v>
+        <v>450</v>
       </c>
       <c r="E9" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>460</v>
+        <v>452</v>
       </c>
       <c r="C10" t="s">
-        <v>461</v>
+        <v>453</v>
       </c>
       <c r="D10" t="s">
-        <v>462</v>
+        <v>454</v>
       </c>
       <c r="E10" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>464</v>
+        <v>456</v>
       </c>
       <c r="C11" t="s">
-        <v>465</v>
+        <v>457</v>
       </c>
       <c r="D11" t="s">
-        <v>466</v>
+        <v>458</v>
       </c>
       <c r="E11" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>468</v>
+        <v>460</v>
       </c>
       <c r="C12" t="s">
-        <v>469</v>
+        <v>461</v>
       </c>
       <c r="D12" t="s">
-        <v>470</v>
+        <v>462</v>
       </c>
       <c r="E12" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>472</v>
+        <v>464</v>
       </c>
       <c r="C13" t="s">
-        <v>473</v>
+        <v>465</v>
       </c>
       <c r="D13" t="s">
-        <v>474</v>
+        <v>466</v>
       </c>
       <c r="E13" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>476</v>
+        <v>468</v>
       </c>
       <c r="C14" t="s">
-        <v>477</v>
+        <v>469</v>
       </c>
       <c r="D14" t="s">
-        <v>478</v>
+        <v>470</v>
       </c>
       <c r="E14" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>480</v>
+        <v>472</v>
       </c>
       <c r="C15" t="s">
-        <v>481</v>
+        <v>473</v>
       </c>
       <c r="D15" t="s">
-        <v>482</v>
+        <v>474</v>
       </c>
       <c r="E15" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>484</v>
+        <v>476</v>
       </c>
       <c r="C16" t="s">
-        <v>485</v>
+        <v>477</v>
       </c>
       <c r="D16" t="s">
-        <v>486</v>
+        <v>478</v>
       </c>
       <c r="E16" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>488</v>
+        <v>480</v>
       </c>
       <c r="C17" t="s">
-        <v>489</v>
+        <v>481</v>
       </c>
       <c r="D17" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="E17" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>492</v>
+        <v>484</v>
       </c>
       <c r="C18" t="s">
-        <v>493</v>
+        <v>485</v>
       </c>
       <c r="D18" t="s">
-        <v>494</v>
+        <v>486</v>
       </c>
       <c r="E18" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
       <c r="C19" t="s">
-        <v>497</v>
+        <v>489</v>
       </c>
       <c r="D19" t="s">
-        <v>498</v>
+        <v>490</v>
       </c>
       <c r="E19" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>500</v>
+        <v>492</v>
       </c>
       <c r="C20" t="s">
-        <v>501</v>
+        <v>493</v>
       </c>
       <c r="D20" t="s">
-        <v>502</v>
+        <v>494</v>
       </c>
       <c r="E20" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>504</v>
+        <v>496</v>
       </c>
       <c r="C21" t="s">
-        <v>505</v>
+        <v>497</v>
       </c>
       <c r="D21" t="s">
-        <v>506</v>
+        <v>498</v>
       </c>
       <c r="E21" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>508</v>
+        <v>500</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>509</v>
+        <v>501</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>510</v>
+        <v>502</v>
       </c>
       <c r="E22" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>512</v>
+        <v>504</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>513</v>
+        <v>505</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>514</v>
+        <v>506</v>
       </c>
       <c r="E23" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>516</v>
+        <v>508</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>517</v>
+        <v>509</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>516</v>
+        <v>508</v>
       </c>
       <c r="E24" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>518</v>
+        <v>510</v>
       </c>
       <c r="C25" t="s">
-        <v>519</v>
+        <v>511</v>
       </c>
       <c r="D25" t="s">
-        <v>520</v>
+        <v>512</v>
       </c>
       <c r="E25" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="C26" t="s">
-        <v>523</v>
+        <v>515</v>
       </c>
       <c r="D26" t="s">
-        <v>524</v>
+        <v>516</v>
       </c>
       <c r="E26" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>526</v>
+        <v>518</v>
       </c>
       <c r="C27" t="s">
-        <v>527</v>
+        <v>519</v>
       </c>
       <c r="D27" t="s">
-        <v>528</v>
+        <v>520</v>
       </c>
       <c r="E27" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>530</v>
+        <v>521</v>
       </c>
       <c r="C28" t="s">
-        <v>531</v>
+        <v>522</v>
       </c>
       <c r="D28" t="s">
-        <v>532</v>
+        <v>523</v>
       </c>
       <c r="E28" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>534</v>
+        <v>525</v>
       </c>
       <c r="C29" t="s">
-        <v>535</v>
+        <v>526</v>
       </c>
       <c r="D29" t="s">
-        <v>536</v>
+        <v>527</v>
       </c>
       <c r="E29" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A30">
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>538</v>
+        <v>529</v>
       </c>
       <c r="C30" t="s">
-        <v>539</v>
+        <v>530</v>
       </c>
       <c r="D30" t="s">
-        <v>540</v>
+        <v>531</v>
       </c>
       <c r="E30" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A31">
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>541</v>
+        <v>532</v>
       </c>
       <c r="C31" t="s">
-        <v>542</v>
+        <v>533</v>
       </c>
       <c r="D31" t="s">
-        <v>543</v>
+        <v>534</v>
       </c>
       <c r="E31" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="14.4" x14ac:dyDescent="0.3">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A32">
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>545</v>
+        <v>536</v>
       </c>
       <c r="C32" t="s">
-        <v>546</v>
+        <v>537</v>
       </c>
       <c r="D32" t="s">
-        <v>547</v>
+        <v>538</v>
       </c>
       <c r="E32" t="s">
-        <v>548</v>
+        <v>539</v>
       </c>
     </row>
   </sheetData>
@@ -5028,9 +5015,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1661D22-A73B-4F85-82EE-7D613C5D43C3}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -5041,112 +5028,112 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>339</v>
+        <v>332</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>549</v>
+        <v>540</v>
       </c>
       <c r="C2" t="s">
-        <v>550</v>
+        <v>541</v>
       </c>
       <c r="D2" t="s">
-        <v>550</v>
+        <v>541</v>
       </c>
       <c r="E2" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>552</v>
+        <v>542</v>
       </c>
       <c r="C3" t="s">
-        <v>553</v>
+        <v>543</v>
       </c>
       <c r="D3" t="s">
-        <v>554</v>
+        <v>544</v>
       </c>
       <c r="E3" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>556</v>
+        <v>588</v>
       </c>
       <c r="C4" t="s">
-        <v>557</v>
+        <v>545</v>
       </c>
       <c r="D4" t="s">
-        <v>558</v>
+        <v>546</v>
       </c>
       <c r="E4" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>559</v>
+        <v>547</v>
       </c>
       <c r="C5" t="s">
-        <v>560</v>
+        <v>548</v>
       </c>
       <c r="D5" t="s">
-        <v>561</v>
+        <v>549</v>
       </c>
       <c r="E5" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>563</v>
+        <v>551</v>
       </c>
       <c r="C6" t="s">
-        <v>564</v>
+        <v>552</v>
       </c>
       <c r="D6" t="s">
-        <v>569</v>
+        <v>556</v>
       </c>
       <c r="E6" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>566</v>
+        <v>554</v>
       </c>
       <c r="C7" t="s">
-        <v>567</v>
+        <v>555</v>
       </c>
       <c r="D7" t="s">
-        <v>567</v>
+        <v>555</v>
       </c>
       <c r="E7" t="s">
-        <v>568</v>
+        <v>554</v>
       </c>
     </row>
   </sheetData>
@@ -5155,6 +5142,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010033C2A0066C18BC4E9BE6DC4E41B0C07F" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="09e1717f508eb245191a7d70af1a5d50">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b" xmlns:ns3="9bae65c2-241c-418a-a37c-ddfb2f921707" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b81c025f9de5594d7b8cbb661cb82c62" ns2:_="" ns3:_="">
     <xsd:import namespace="0d50eb87-dd2c-4cc8-80b9-5e27a2995b6b"/>
@@ -5415,15 +5411,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5436,6 +5423,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309E3272-FC41-444B-BA86-D1A5622D221C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97FE3D86-31EC-465E-A8A6-6E0CEA7D99AC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5454,14 +5449,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{309E3272-FC41-444B-BA86-D1A5622D221C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E773F732-AD26-4990-9766-F75C55FCDDD2}">
   <ds:schemaRefs>

</xml_diff>